<commit_message>
Actualiza informe APA y métricas de interoperabilidad
</commit_message>
<xml_diff>
--- a/MEDICION ISO/ISO25023-Mediciones-Interoperabilidad-ToleranciaFallos.xlsx
+++ b/MEDICION ISO/ISO25023-Mediciones-Interoperabilidad-ToleranciaFallos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3f28f189b2c0b5/Documentos/integracion/RESTAURANT/Restaurants/MEDICION ISO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026 - I\Integración de sistemas de soft\RESTAURANTES SUBIDOS\Restaurants\MEDICION ISO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_2BA7764121F7A2FD4A2AB743243ED3128643B52B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28BAD5C1-5075-4DAD-8D01-F78B107089C9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5B0B42-93B1-435E-9CEC-5026065216CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -447,13 +447,13 @@
     <t>Producción: Vercel — edge/CDN multi-nodo gestionado</t>
   </si>
   <si>
-    <t xml:space="preserve">Interoperabilidad: medición 2026-07-04. Tolerancia a fallos: PRIMERA EJECUCIÓN 2026-07-05 </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Criterios: docs/interoperabilidad.md</t>
   </si>
   <si>
     <t xml:space="preserve"> Fuente: resultados/tolerancia a fallos/primera_ejecucion/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interoperabilidad: medición 2026-07-04. Tolerancia a fallos: PRIMERA EJECUCIÓN 2026-07-07 </t>
   </si>
 </sst>
 </file>
@@ -589,12 +589,6 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -622,6 +616,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1019,345 +1019,345 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>131</v>
+      <c r="A2" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <f>COUNTIFS('Datos Interoperabilidad'!A5:A20,"CIn-1-G",'Datos Interoperabilidad'!E5:E20,"INTERCAMBIABLE")</f>
         <v>3</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <f>COUNTIF('Datos Interoperabilidad'!A5:A20,"CIn-1-G")</f>
         <v>3</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="7">
         <f>E6/F6</f>
         <v>1</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <f>IF(G6&gt;=0.9,"CUMPLE",IF(G6&gt;=0.7,"PARCIAL","NO CUMPLE"))</f>
         <v>CUMPLE</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <f>COUNTIFS('Datos Interoperabilidad'!A5:A20,"CIn-2-G",'Datos Interoperabilidad'!E5:E20,"SOPORTADO")</f>
         <v>3</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="4">
         <f>COUNTIF('Datos Interoperabilidad'!A5:A20,"CIn-2-G")</f>
         <v>3</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="7">
         <f>E7/F7</f>
         <v>1</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <f>IF(G7&gt;=0.9,"CUMPLE",IF(G7&gt;=0.7,"PARCIAL","NO CUMPLE"))</f>
         <v>CUMPLE</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <f>COUNTIFS('Datos Interoperabilidad'!A5:A20,"CIn-3-S",'Datos Interoperabilidad'!E5:E20,"FUNCIONAL")</f>
         <v>3</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="4">
         <f>COUNTIF('Datos Interoperabilidad'!A5:A20,"CIn-3-S")</f>
         <v>3</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="7">
         <f>E8/F8</f>
         <v>1</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <f>IF(G8&gt;=0.9,"CUMPLE",IF(G8&gt;=0.7,"PARCIAL","NO CUMPLE"))</f>
         <v>CUMPLE</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="11" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="4">
         <f>COUNTIF('Datos Casos de fallo'!F5:F40,"EVITADO")</f>
         <v>6</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="4">
         <f>COUNTA('Datos Casos de fallo'!F5:F40)</f>
         <v>12</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="7">
         <f>E13/F13</f>
         <v>0.5</v>
       </c>
-      <c r="H13" s="6" t="str">
+      <c r="H13" s="4" t="str">
         <f>IF(G13&gt;=0.9,"CUMPLE",IF(G13&gt;=0.7,"PARCIAL","NO CUMPLE"))</f>
         <v>NO CUMPLE</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="4">
         <f>COUNTIF('Datos Componentes'!C5:C20,"SI")</f>
         <v>0</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="4">
         <f>COUNTA('Datos Componentes'!C5:C20)</f>
         <v>3</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="7">
         <f>E14/F14</f>
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="str">
+      <c r="H14" s="4" t="str">
         <f>IF(G14&gt;=0.9,"CUMPLE",IF(G14&gt;=0.7,"PARCIAL","NO CUMPLE"))</f>
         <v>NO CUMPLE</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="4">
         <f>COUNTIF('Datos Componentes'!D5:D20,"SI")</f>
         <v>2</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="4">
         <f>COUNTA('Datos Componentes'!D5:D20)</f>
         <v>3</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="7">
         <f>E15/F15</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="H15" s="6" t="str">
+      <c r="H15" s="4" t="str">
         <f>IF(G15&gt;=0.9,"CUMPLE",IF(G15&gt;=0.7,"PARCIAL","NO CUMPLE"))</f>
         <v>NO CUMPLE</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" ht="96" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="4">
         <f>SUM('Datos Casos de fallo'!H5:H40)</f>
         <v>0.95300000000000007</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="4">
         <f>COUNT('Datos Casos de fallo'!H5:H40)</f>
         <v>12</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="8">
         <f>E17/F17</f>
         <v>7.9416666666666677E-2</v>
       </c>
-      <c r="H17" s="6" t="str">
+      <c r="H17" s="4" t="str">
         <f>IF(G17&lt;=1,"CUMPLE","NO CUMPLE")</f>
         <v>CUMPLE</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="20" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4"/>
+      <c r="A20" s="2"/>
     </row>
     <row r="21" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4"/>
+      <c r="A21" s="2"/>
     </row>
     <row r="22" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="4"/>
+      <c r="A22" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1451,212 +1451,212 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>132</v>
+      <c r="A2" s="2" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="6" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="6" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="6" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="6" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="6" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1688,350 +1688,350 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>133</v>
+      <c r="A2" s="2" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="3" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <v>1</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="6">
         <v>500</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="10">
         <v>0.24199999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="A6" s="6">
         <v>2</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="6">
         <v>400</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="10">
         <v>9.4E-2</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <v>3</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="6">
         <v>401</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="10">
         <v>0.40799999999999997</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8">
+      <c r="A8" s="6">
         <v>4</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="6">
         <v>404</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="10">
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
+      <c r="A9" s="6">
         <v>5</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <v>500</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="10">
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8">
+      <c r="A10" s="6">
         <v>6</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="6">
         <v>403</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="10">
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8">
+      <c r="A11" s="6">
         <v>7</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="6">
         <v>403</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="10">
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
+      <c r="A12" s="6">
         <v>8</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="6">
         <v>403</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="10">
         <v>9.8000000000000004E-2</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8">
+      <c r="A13" s="6">
         <v>9</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="6">
         <v>500</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="10">
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8">
+      <c r="A14" s="6">
         <v>10</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14" s="6">
         <v>500</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="10">
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8">
+      <c r="A15" s="6">
         <v>11</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="6">
         <v>500</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="10">
         <v>0.02</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8">
+      <c r="A16" s="6">
         <v>12</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="6">
         <v>500</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="10">
         <v>0.01</v>
       </c>
     </row>
@@ -2060,84 +2060,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
+      <c r="A2" s="2"/>
     </row>
     <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="3" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="6">
         <v>1</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="6">
         <v>1</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="6" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="6">
         <v>1</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="6" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D13" s="13"/>
+      <c r="D13" s="11"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
feat: add comun.ps1 script with helper functions for HTTP measurement, authentication, and CSV logging
</commit_message>
<xml_diff>
--- a/MEDICION ISO/ISO25023-Mediciones-Interoperabilidad-ToleranciaFallos.xlsx
+++ b/MEDICION ISO/ISO25023-Mediciones-Interoperabilidad-ToleranciaFallos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026 - I\Integración de sistemas de soft\RESTAURANTES SUBIDOS\Restaurants\MEDICION ISO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3f28f189b2c0b5/Documentos/integracion/RESTAURANT/Restaurants/MEDICION ISO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5B0B42-93B1-435E-9CEC-5026065216CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{DE5B0B42-93B1-435E-9CEC-5026065216CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A583B19A-517B-43A3-B6B7-89A24B964536}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -453,7 +453,7 @@
     <t xml:space="preserve"> Fuente: resultados/tolerancia a fallos/primera_ejecucion/</t>
   </si>
   <si>
-    <t xml:space="preserve">Interoperabilidad: medición 2026-07-04. Tolerancia a fallos: PRIMERA EJECUCIÓN 2026-07-07 </t>
+    <t xml:space="preserve">Interoperabilidad: medición 2026-07-07. Tolerancia a fallos: PRIMERA EJECUCIÓN 2026-07-07 </t>
   </si>
 </sst>
 </file>

</xml_diff>